<commit_message>
cicada IG: refresh the site copy from build 18 (0 errors, 0 warnings)
Built with publisher 2.3.4 from cicada 08df1b0f, 2026-09-07.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014oU3PKgtLkXXkkKZoLLRok
</commit_message>
<xml_diff>
--- a/jaspr/web/cicada_ig/StructureDefinition-begin-age.xlsx
+++ b/jaspr/web/cicada_ig/StructureDefinition-begin-age.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-07T19:28:06-04:00</t>
+    <t>2026-09-07T19:51:55-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -129,7 +129,7 @@
     <t>Context</t>
   </si>
   <si>
-    <t>element:Element</t>
+    <t>element:Medication</t>
   </si>
   <si>
     <t>ID</t>

</xml_diff>